<commit_message>
fixed repo names and added filtering for .tsv files in fetch_scores.py, updated imports and variable names in myself.py to reflect changes.
</commit_message>
<xml_diff>
--- a/Docs/2.02.26/BWV1001_Martin_system.xlsx
+++ b/Docs/2.02.26/BWV1001_Martin_system.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding\TAU-RA-Code\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Coding\TAU-RA-Code\docs\2.02.26\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162227CA-7FBD-42B6-8F42-951BA8D9EE44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4352B3A9-6BAF-4843-A303-758EEE5D1432}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{3137263C-90DF-44F5-B689-225A2B9B7652}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>mc</t>
   </si>
@@ -71,48 +71,6 @@
     <t>label</t>
   </si>
   <si>
-    <t>globalkey</t>
-  </si>
-  <si>
-    <t>localkey</t>
-  </si>
-  <si>
-    <t>pedal</t>
-  </si>
-  <si>
-    <t>chord</t>
-  </si>
-  <si>
-    <t>numeral</t>
-  </si>
-  <si>
-    <t>form</t>
-  </si>
-  <si>
-    <t>figbass</t>
-  </si>
-  <si>
-    <t>changes</t>
-  </si>
-  <si>
-    <t>relativeroot</t>
-  </si>
-  <si>
-    <t>cadence</t>
-  </si>
-  <si>
-    <t>phraseend</t>
-  </si>
-  <si>
-    <t>chord_type</t>
-  </si>
-  <si>
-    <t>globalkey_is_minor</t>
-  </si>
-  <si>
-    <t>localkey_is_minor</t>
-  </si>
-  <si>
     <t>chord_tones</t>
   </si>
   <si>
@@ -125,18 +83,6 @@
     <t>g.i{</t>
   </si>
   <si>
-    <t>g</t>
-  </si>
-  <si>
-    <t>i</t>
-  </si>
-  <si>
-    <t>{</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
     <t>1, -2, 2</t>
   </si>
   <si>
@@ -146,12 +92,6 @@
     <t>#viio6(2)</t>
   </si>
   <si>
-    <t>#vii</t>
-  </si>
-  <si>
-    <t>o</t>
-  </si>
-  <si>
     <t>3, 0, 1</t>
   </si>
   <si>
@@ -164,40 +104,25 @@
     <t>V</t>
   </si>
   <si>
-    <t>M</t>
-  </si>
-  <si>
     <t>2, 6, 3</t>
   </si>
   <si>
     <t>V7</t>
   </si>
   <si>
-    <t>Mm7</t>
-  </si>
-  <si>
     <t>2, 6, 3, 0</t>
   </si>
   <si>
     <t>i}</t>
   </si>
   <si>
-    <t>}</t>
-  </si>
-  <si>
     <t>VI6</t>
   </si>
   <si>
-    <t>VI</t>
-  </si>
-  <si>
     <t>1, -2, -3</t>
   </si>
   <si>
     <t>v6(2)</t>
-  </si>
-  <si>
-    <t>v</t>
   </si>
   <si>
     <t>-1, 3, -3</t>
@@ -1071,7 +996,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F1B5E0DC-A04F-4918-A728-AE8BDACED963}">
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:P11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -1079,7 +1004,7 @@
     <col min="10" max="10" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1108,7 +1033,7 @@
         <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="K1" t="s">
         <v>9</v>
@@ -1128,50 +1053,8 @@
       <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="Q1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" t="s">
-        <v>20</v>
-      </c>
-      <c r="W1" t="s">
-        <v>21</v>
-      </c>
-      <c r="X1" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>26</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>27</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>28</v>
-      </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1197,45 +1080,21 @@
         <v>1</v>
       </c>
       <c r="M2" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="N2" t="s">
-        <v>30</v>
-      </c>
-      <c r="O2" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>31</v>
-      </c>
-      <c r="R2" t="s">
-        <v>31</v>
-      </c>
-      <c r="X2" t="s">
-        <v>32</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z2">
-        <v>1</v>
-      </c>
-      <c r="AA2">
-        <v>1</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>34</v>
-      </c>
-      <c r="AD2">
+        <v>16</v>
+      </c>
+      <c r="P2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="C3">
         <v>0.5</v>
@@ -1268,46 +1127,16 @@
         <v>1</v>
       </c>
       <c r="M3" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="N3" t="s">
-        <v>30</v>
-      </c>
-      <c r="O3" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>36</v>
-      </c>
-      <c r="R3" t="s">
-        <v>37</v>
-      </c>
-      <c r="S3" t="s">
-        <v>38</v>
-      </c>
-      <c r="T3">
-        <v>6</v>
-      </c>
-      <c r="U3">
-        <v>2</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z3">
-        <v>1</v>
-      </c>
-      <c r="AA3">
-        <v>1</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD3">
+        <v>19</v>
+      </c>
+      <c r="P3">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1318,7 +1147,7 @@
         <v>0.625</v>
       </c>
       <c r="D4">
-        <f t="shared" ref="D4:D10" si="0">(C4-C3)+(A4-A3)*F3</f>
+        <f>(C4-C3)+(A4-A3)*F3</f>
         <v>0.125</v>
       </c>
       <c r="E4" s="1">
@@ -1331,15 +1160,15 @@
         <v>6</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H4:H10" si="1">G4-G3</f>
+        <f t="shared" ref="H4:H10" si="0">G4-G3</f>
         <v>0</v>
       </c>
       <c r="I4">
-        <f t="shared" ref="I4:I9" si="2">D4+D5</f>
+        <f t="shared" ref="I4:I8" si="1">D4+D5</f>
         <v>0.25</v>
       </c>
       <c r="J4">
-        <f>I4+I3</f>
+        <f t="shared" ref="J4:J10" si="2">I4+I3</f>
         <v>0.875</v>
       </c>
       <c r="K4">
@@ -1349,43 +1178,16 @@
         <v>1</v>
       </c>
       <c r="M4" t="s">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="N4" t="s">
-        <v>30</v>
-      </c>
-      <c r="O4" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>40</v>
-      </c>
-      <c r="R4" t="s">
-        <v>37</v>
-      </c>
-      <c r="S4" t="s">
-        <v>38</v>
-      </c>
-      <c r="T4">
-        <v>6</v>
-      </c>
-      <c r="Y4" t="s">
-        <v>38</v>
-      </c>
-      <c r="Z4">
-        <v>1</v>
-      </c>
-      <c r="AA4">
-        <v>1</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>41</v>
-      </c>
-      <c r="AD4">
+        <v>21</v>
+      </c>
+      <c r="P4">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1396,7 +1198,7 @@
         <v>0.75</v>
       </c>
       <c r="D5">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="D5:D10" si="3">(C5-C4)+(A5-A4)*F4</f>
         <v>0.125</v>
       </c>
       <c r="E5" s="1">
@@ -1409,15 +1211,15 @@
         <v>2</v>
       </c>
       <c r="H5">
+        <f t="shared" si="0"/>
+        <v>-4</v>
+      </c>
+      <c r="I5">
         <f t="shared" si="1"/>
-        <v>-4</v>
-      </c>
-      <c r="I5">
+        <v>0.375</v>
+      </c>
+      <c r="J5">
         <f t="shared" si="2"/>
-        <v>0.375</v>
-      </c>
-      <c r="J5">
-        <f>I5+I4</f>
         <v>0.625</v>
       </c>
       <c r="K5">
@@ -1427,37 +1229,16 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="N5" t="s">
-        <v>30</v>
-      </c>
-      <c r="O5" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>42</v>
-      </c>
-      <c r="R5" t="s">
-        <v>42</v>
-      </c>
-      <c r="Y5" t="s">
-        <v>43</v>
-      </c>
-      <c r="Z5">
-        <v>1</v>
-      </c>
-      <c r="AA5">
-        <v>1</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>44</v>
-      </c>
-      <c r="AD5">
+        <v>23</v>
+      </c>
+      <c r="P5">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2</v>
       </c>
@@ -1468,7 +1249,7 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.25</v>
       </c>
       <c r="E6" s="1">
@@ -1481,15 +1262,15 @@
         <v>2</v>
       </c>
       <c r="H6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I6">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="I6">
+        <v>0.75</v>
+      </c>
+      <c r="J6">
         <f t="shared" si="2"/>
-        <v>0.75</v>
-      </c>
-      <c r="J6">
-        <f>I6+I5</f>
         <v>1.125</v>
       </c>
       <c r="K6">
@@ -1499,40 +1280,16 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="N6" t="s">
-        <v>30</v>
-      </c>
-      <c r="O6" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>45</v>
-      </c>
-      <c r="R6" t="s">
-        <v>42</v>
-      </c>
-      <c r="T6">
-        <v>7</v>
-      </c>
-      <c r="Y6" t="s">
-        <v>46</v>
-      </c>
-      <c r="Z6">
-        <v>1</v>
-      </c>
-      <c r="AA6">
-        <v>1</v>
-      </c>
-      <c r="AB6" t="s">
-        <v>47</v>
-      </c>
-      <c r="AD6">
+        <v>25</v>
+      </c>
+      <c r="P6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2</v>
       </c>
@@ -1543,7 +1300,7 @@
         <v>0.5</v>
       </c>
       <c r="D7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.5</v>
       </c>
       <c r="E7" s="1">
@@ -1556,15 +1313,15 @@
         <v>1</v>
       </c>
       <c r="H7">
+        <f t="shared" si="0"/>
+        <v>-1</v>
+      </c>
+      <c r="I7">
         <f t="shared" si="1"/>
-        <v>-1</v>
-      </c>
-      <c r="I7">
+        <v>0.75</v>
+      </c>
+      <c r="J7">
         <f t="shared" si="2"/>
-        <v>0.75</v>
-      </c>
-      <c r="J7">
-        <f>I7+I6</f>
         <v>1.5</v>
       </c>
       <c r="K7">
@@ -1574,40 +1331,16 @@
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="N7" t="s">
-        <v>30</v>
-      </c>
-      <c r="O7" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>31</v>
-      </c>
-      <c r="R7" t="s">
-        <v>31</v>
-      </c>
-      <c r="X7" t="s">
-        <v>49</v>
-      </c>
-      <c r="Y7" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z7">
-        <v>1</v>
-      </c>
-      <c r="AA7">
-        <v>1</v>
-      </c>
-      <c r="AB7" t="s">
-        <v>34</v>
-      </c>
-      <c r="AD7">
+        <v>16</v>
+      </c>
+      <c r="P7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2</v>
       </c>
@@ -1618,7 +1351,7 @@
         <v>0.75</v>
       </c>
       <c r="D8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.25</v>
       </c>
       <c r="E8" s="1">
@@ -1631,15 +1364,15 @@
         <v>-3</v>
       </c>
       <c r="H8">
+        <f t="shared" si="0"/>
+        <v>-4</v>
+      </c>
+      <c r="I8">
         <f t="shared" si="1"/>
-        <v>-4</v>
-      </c>
-      <c r="I8">
+        <v>0.5</v>
+      </c>
+      <c r="J8">
         <f t="shared" si="2"/>
-        <v>0.5</v>
-      </c>
-      <c r="J8">
-        <f>I8+I7</f>
         <v>1.25</v>
       </c>
       <c r="K8">
@@ -1649,40 +1382,16 @@
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="N8" t="s">
-        <v>30</v>
-      </c>
-      <c r="O8" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q8" t="s">
-        <v>50</v>
-      </c>
-      <c r="R8" t="s">
-        <v>51</v>
-      </c>
-      <c r="T8">
-        <v>6</v>
-      </c>
-      <c r="Y8" t="s">
-        <v>43</v>
-      </c>
-      <c r="Z8">
-        <v>1</v>
-      </c>
-      <c r="AA8">
-        <v>1</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>52</v>
-      </c>
-      <c r="AD8">
+        <v>28</v>
+      </c>
+      <c r="P8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>3</v>
       </c>
@@ -1693,7 +1402,7 @@
         <v>0</v>
       </c>
       <c r="D9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.25</v>
       </c>
       <c r="E9" s="1">
@@ -1706,7 +1415,7 @@
         <v>2</v>
       </c>
       <c r="H9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="I9">
@@ -1714,7 +1423,7 @@
         <v>0.5</v>
       </c>
       <c r="J9">
-        <f>I9+I8</f>
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
       <c r="K9">
@@ -1724,43 +1433,16 @@
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="N9" t="s">
         <v>30</v>
       </c>
-      <c r="O9" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>53</v>
-      </c>
-      <c r="R9" t="s">
-        <v>54</v>
-      </c>
-      <c r="T9">
-        <v>6</v>
-      </c>
-      <c r="U9">
-        <v>2</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z9">
-        <v>1</v>
-      </c>
-      <c r="AA9">
-        <v>1</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>55</v>
-      </c>
-      <c r="AD9">
+      <c r="P9">
         <v>-1</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>3</v>
       </c>
@@ -1771,7 +1453,7 @@
         <v>0.25</v>
       </c>
       <c r="D10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>0.25</v>
       </c>
       <c r="E10" s="1">
@@ -1784,7 +1466,7 @@
         <v>2</v>
       </c>
       <c r="H10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="I10">
@@ -1792,7 +1474,7 @@
         <v>0.25</v>
       </c>
       <c r="J10">
-        <f>I10+I9</f>
+        <f t="shared" si="2"/>
         <v>0.75</v>
       </c>
       <c r="K10">
@@ -1802,40 +1484,16 @@
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="N10" t="s">
-        <v>30</v>
-      </c>
-      <c r="O10" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>56</v>
-      </c>
-      <c r="R10" t="s">
-        <v>54</v>
-      </c>
-      <c r="T10">
-        <v>6</v>
-      </c>
-      <c r="Y10" t="s">
-        <v>33</v>
-      </c>
-      <c r="Z10">
-        <v>1</v>
-      </c>
-      <c r="AA10">
-        <v>1</v>
-      </c>
-      <c r="AB10" t="s">
-        <v>57</v>
-      </c>
-      <c r="AD10">
+        <v>32</v>
+      </c>
+      <c r="P10">
         <v>-1</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C11">
         <v>0</v>
       </c>

</xml_diff>